<commit_message>
latest jan 2026 file
</commit_message>
<xml_diff>
--- a/data/boprc_cyano/og_excel_files/Cyanobacteria Report-20260108.xlsx
+++ b/data/boprc_cyano/og_excel_files/Cyanobacteria Report-20260108.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://boprc-my.sharepoint.com/personal/amber_sutherland_boprc_govt_nz/Documents/Desktop/Amber Sutherland 2025-2026/Cyanobacteria weekly results 2025-2026/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://waikatouniversitynz-my.sharepoint.com/personal/whitney_woelmer_waikato_ac_nz/Documents/Desktop/lakecast_rotorua/data/boprc_cyano/og_excel_files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC2CED31-B908-44A0-A282-3220D474C2BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="8_{AC2CED31-B908-44A0-A282-3220D474C2BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DEF76A1F-2B61-44F1-A063-03EA844A1525}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Lakes Data" sheetId="2" r:id="rId1"/>
@@ -387,7 +387,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -463,25 +463,26 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1">
+  <cellXfs count="12">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="169" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="169" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="169" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" pivotButton="1"/>
+    <xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="17">
+  <dxfs count="24">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -490,22 +491,87 @@
       </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="168" formatCode="0.0000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="169" formatCode="0.000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF99FF33"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="0.00000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF99FF33"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="166" formatCode="0.000000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF99FF33"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0000000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
     </dxf>
     <dxf>
-      <numFmt numFmtId="164" formatCode="0.00000000"/>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFFC000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF99FF33"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
     </dxf>
     <dxf>
       <fill>
@@ -596,7 +662,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Amber Sutherland" refreshedDate="46030.431794212964" refreshedVersion="8" recordCount="44" xr:uid="{00000000-000A-0000-FFFF-FFFF02000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="46037.471903819445" refreshedVersion="8" recordCount="44" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P45" sheet="Lakes Data"/>
   </cacheSource>
@@ -681,7 +747,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Amber Sutherland" refreshedDate="46030.431794675926" refreshedVersion="8" recordCount="4" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="46037.471904050923" refreshedVersion="8" recordCount="4" xr:uid="{00000000-000A-0000-FFFF-FFFF01000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P5" sheet="Toxin Data"/>
   </cacheSource>
@@ -758,7 +824,7 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Amber Sutherland" refreshedDate="46030.43179490741" refreshedVersion="8" recordCount="44" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Whitney Woelmer" refreshedDate="46037.471904282407" refreshedVersion="8" recordCount="44" xr:uid="{00000000-000A-0000-FFFF-FFFF02000000}">
   <cacheSource type="worksheet">
     <worksheetSource ref="A1:P45" sheet="Lakes Data"/>
   </cacheSource>
@@ -2514,7 +2580,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="AlertWarning" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="AlertWarning" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
   <location ref="A8:D23" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
   <pivotFields count="16">
     <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
@@ -2630,7 +2696,7 @@
     <dataField name="PotentiallyToxicBioVolume" fld="14" baseField="0" baseItem="0"/>
   </dataFields>
   <formats count="11">
-    <format dxfId="16">
+    <format dxfId="23">
       <pivotArea outline="0" fieldPosition="0">
         <references count="1">
           <reference field="1" count="1" selected="0">
@@ -2639,7 +2705,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="15">
+    <format dxfId="22">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="1" count="1" selected="0">
@@ -2651,7 +2717,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="21">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="1" count="1" selected="0">
@@ -2665,7 +2731,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="13">
+    <format dxfId="20">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="1" count="1" selected="0">
@@ -2677,7 +2743,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="12">
+    <format dxfId="19">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="1" count="1" selected="0">
@@ -2689,7 +2755,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="11">
+    <format dxfId="18">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="1" count="1" selected="0">
@@ -2701,7 +2767,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="10">
+    <format dxfId="17">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="1" count="1" selected="0">
@@ -2715,7 +2781,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="9">
+    <format dxfId="16">
       <pivotArea outline="0" fieldPosition="0">
         <references count="2">
           <reference field="1" count="1" selected="0">
@@ -2727,7 +2793,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="8">
+    <format dxfId="15">
       <pivotArea outline="0" fieldPosition="0">
         <references count="4">
           <reference field="4294967294" count="1" selected="0">
@@ -2743,7 +2809,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="7">
+    <format dxfId="14">
       <pivotArea outline="0" fieldPosition="0">
         <references count="4">
           <reference field="4294967294" count="1" selected="0">
@@ -2759,7 +2825,7 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="2">
+    <format dxfId="13">
       <pivotArea outline="0" fieldPosition="0"/>
     </format>
   </formats>
@@ -2773,98 +2839,7 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000002000000}" name="CellsPermL" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
-  <location ref="A8:D14" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
-  <pivotFields count="16">
-    <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Location" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-      </items>
-    </pivotField>
-    <pivotField name="Site" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="4">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-      </items>
-    </pivotField>
-    <pivotField name="Dates" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="1">
-        <item x="0"/>
-      </items>
-    </pivotField>
-    <pivotField name="MicroscopeType" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="WholePlate" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Species" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="IsSpeciesToxic" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="VolumeInMillilitres" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="Average" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="NumberOfColonies" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="CellsPerMl" dataField="1" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="TotalBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="PotentiallyToxicCellMl" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="PotentiallyToxicBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
-    <pivotField name="ToxinCluster" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
-      <items count="2">
-        <item m="1" x="1"/>
-        <item x="0"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="2">
-    <field x="1"/>
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="4">
-    <i>
-      <x/>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-      <x v="1"/>
-    </i>
-    <i r="1">
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="2"/>
-      <x v="2"/>
-    </i>
-  </rowItems>
-  <colFields count="2">
-    <field x="3"/>
-    <field x="15"/>
-  </colFields>
-  <colItems count="1">
-    <i>
-      <x/>
-      <x v="1"/>
-    </i>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="CellsPerMl" fld="11" baseField="0" baseItem="0"/>
-  </dataFields>
-  <formats count="1">
-    <format dxfId="0">
-      <pivotArea outline="0" fieldPosition="0"/>
-    </format>
-  </formats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="AlertWarning" cacheId="8" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000001000000}" name="AlertWarning" cacheId="21" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
   <location ref="A37:C51" firstHeaderRow="1" firstDataRow="2" firstDataCol="2"/>
   <pivotFields count="16">
     <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
@@ -2973,6 +2948,97 @@
   <dataFields count="1">
     <dataField name="TotalBioVolume" fld="12" baseField="0" baseItem="0"/>
   </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
+  <extLst>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0300-000002000000}" name="CellsPermL" cacheId="15" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="Values" missingCaption="" updatedVersion="8" rowGrandTotals="0" colGrandTotals="0" compact="0" compactData="0" gridDropZones="1" rowHeaderCaption="Locations" colHeaderCaption="Dates">
+  <location ref="A8:D14" firstHeaderRow="1" firstDataRow="3" firstDataCol="2"/>
+  <pivotFields count="16">
+    <pivotField name="SampleId" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Location" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+      </items>
+    </pivotField>
+    <pivotField name="Site" axis="axisRow" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="4">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+      </items>
+    </pivotField>
+    <pivotField name="Dates" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="1">
+        <item x="0"/>
+      </items>
+    </pivotField>
+    <pivotField name="MicroscopeType" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="WholePlate" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Species" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="IsSpeciesToxic" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="VolumeInMillilitres" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="Average" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="NumberOfColonies" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="CellsPerMl" dataField="1" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="TotalBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="PotentiallyToxicCellMl" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="PotentiallyToxicBioVolume" compact="0" outline="0" defaultSubtotal="0"/>
+    <pivotField name="ToxinCluster" axis="axisCol" compact="0" outline="0" showAll="0" defaultSubtotal="0">
+      <items count="2">
+        <item m="1" x="1"/>
+        <item x="0"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="2">
+    <field x="1"/>
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="4">
+    <i>
+      <x/>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+      <x v="1"/>
+    </i>
+    <i r="1">
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="2"/>
+      <x v="2"/>
+    </i>
+  </rowItems>
+  <colFields count="2">
+    <field x="3"/>
+    <field x="15"/>
+  </colFields>
+  <colItems count="1">
+    <i>
+      <x/>
+      <x v="1"/>
+    </i>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="CellsPerMl" fld="11" baseField="0" baseItem="0"/>
+  </dataFields>
+  <formats count="1">
+    <format dxfId="12">
+      <pivotArea outline="0" fieldPosition="0"/>
+    </format>
+  </formats>
   <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="0"/>
   <extLst>
     <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
@@ -3318,27 +3384,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:P45"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.453125" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" customWidth="1"/>
-    <col min="3" max="3" width="13.81640625" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" customWidth="1"/>
-    <col min="5" max="5" width="18.6328125" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="32.1796875" customWidth="1"/>
-    <col min="8" max="8" width="16.6328125" customWidth="1"/>
-    <col min="9" max="9" width="20.7265625" customWidth="1"/>
-    <col min="10" max="10" width="18.26953125" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" customWidth="1"/>
-    <col min="12" max="12" width="18.26953125" customWidth="1"/>
-    <col min="13" max="13" width="22.54296875" customWidth="1"/>
-    <col min="14" max="14" width="23.453125" customWidth="1"/>
-    <col min="15" max="15" width="27.36328125" customWidth="1"/>
-    <col min="16" max="16" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="12.47265625" customWidth="1"/>
+    <col min="2" max="2" width="11.7890625" customWidth="1"/>
+    <col min="3" max="3" width="13.7890625" customWidth="1"/>
+    <col min="4" max="4" width="14.7890625" customWidth="1"/>
+    <col min="5" max="5" width="18.62890625" customWidth="1"/>
+    <col min="6" max="6" width="14.47265625" customWidth="1"/>
+    <col min="7" max="7" width="32.15625" customWidth="1"/>
+    <col min="8" max="8" width="16.62890625" customWidth="1"/>
+    <col min="9" max="9" width="20.734375" customWidth="1"/>
+    <col min="10" max="10" width="18.26171875" customWidth="1"/>
+    <col min="11" max="11" width="20.7890625" customWidth="1"/>
+    <col min="12" max="12" width="18.26171875" customWidth="1"/>
+    <col min="13" max="13" width="22.5234375" customWidth="1"/>
+    <col min="14" max="14" width="23.47265625" customWidth="1"/>
+    <col min="15" max="15" width="27.3671875" customWidth="1"/>
+    <col min="16" max="16" width="15.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3388,7 +3454,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>16</v>
       </c>
@@ -3432,7 +3498,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>23</v>
       </c>
@@ -3476,7 +3542,7 @@
         <v>0.468383117475</v>
       </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -3520,7 +3586,7 @@
         <v>8.1367368055555694E-2</v>
       </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -3564,7 +3630,7 @@
         <v>0.234802976388889</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A6" t="s">
         <v>29</v>
       </c>
@@ -3608,7 +3674,7 @@
         <v>0.13744060590000001</v>
       </c>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A7" t="s">
         <v>30</v>
       </c>
@@ -3652,7 +3718,7 @@
         <v>1.98548944444445E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -3696,7 +3762,7 @@
         <v>0.90421451249999896</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -3740,7 +3806,7 @@
         <v>0.66372524513888898</v>
       </c>
     </row>
-    <row r="10" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" t="s">
         <v>36</v>
       </c>
@@ -3787,7 +3853,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -3834,7 +3900,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>42</v>
       </c>
@@ -3881,7 +3947,7 @@
         <v>0.4061331225</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" t="s">
         <v>44</v>
       </c>
@@ -3925,7 +3991,7 @@
         <v>6.94292986111111E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>46</v>
       </c>
@@ -3969,7 +4035,7 @@
         <v>2.2870827777777801E-4</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" t="s">
         <v>48</v>
       </c>
@@ -4013,7 +4079,7 @@
         <v>1.30690444444445E-2</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>50</v>
       </c>
@@ -4057,7 +4123,7 @@
         <v>7.78801951388889E-2</v>
       </c>
     </row>
-    <row r="17" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A17" t="s">
         <v>51</v>
       </c>
@@ -4101,7 +4167,7 @@
         <v>2.7796852222222199E-2</v>
       </c>
     </row>
-    <row r="18" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" t="s">
         <v>53</v>
       </c>
@@ -4145,7 +4211,7 @@
         <v>0.87527964810000303</v>
       </c>
     </row>
-    <row r="19" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A19" t="s">
         <v>54</v>
       </c>
@@ -4189,7 +4255,7 @@
         <v>0.64380073289999895</v>
       </c>
     </row>
-    <row r="20" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>56</v>
       </c>
@@ -4233,7 +4299,7 @@
         <v>5.34699847222221E-2</v>
       </c>
     </row>
-    <row r="21" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" t="s">
         <v>57</v>
       </c>
@@ -4277,7 +4343,7 @@
         <v>0.145393119444445</v>
       </c>
     </row>
-    <row r="22" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>60</v>
       </c>
@@ -4324,7 +4390,7 @@
         <v>3.90846723028125</v>
       </c>
     </row>
-    <row r="23" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>61</v>
       </c>
@@ -4368,7 +4434,7 @@
         <v>6.7418676388888904E-2</v>
       </c>
     </row>
-    <row r="24" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A24" t="s">
         <v>62</v>
       </c>
@@ -4412,7 +4478,7 @@
         <v>0.62209958459999704</v>
       </c>
     </row>
-    <row r="25" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A25" t="s">
         <v>65</v>
       </c>
@@ -4459,7 +4525,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="26" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A26" t="s">
         <v>67</v>
       </c>
@@ -4503,7 +4569,7 @@
         <v>3.9521293055555698E-2</v>
       </c>
     </row>
-    <row r="27" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A27" t="s">
         <v>68</v>
       </c>
@@ -4547,7 +4613,7 @@
         <v>1.88621497222222E-2</v>
       </c>
     </row>
-    <row r="28" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A28" t="s">
         <v>70</v>
       </c>
@@ -4591,7 +4657,7 @@
         <v>0.58231414605000298</v>
       </c>
     </row>
-    <row r="29" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A29" t="s">
         <v>71</v>
       </c>
@@ -4635,7 +4701,7 @@
         <v>9.2991277777777895E-2</v>
       </c>
     </row>
-    <row r="30" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" t="s">
         <v>72</v>
       </c>
@@ -4682,7 +4748,7 @@
         <v>1.5769999999999999E-2</v>
       </c>
     </row>
-    <row r="31" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" t="s">
         <v>75</v>
       </c>
@@ -4729,7 +4795,7 @@
         <v>1.5769999999999999E-2</v>
       </c>
     </row>
-    <row r="32" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" t="s">
         <v>76</v>
       </c>
@@ -4773,7 +4839,7 @@
         <v>1.1839999999999999E-3</v>
       </c>
     </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" t="s">
         <v>77</v>
       </c>
@@ -4817,7 +4883,7 @@
         <v>2.3699999999999999E-4</v>
       </c>
     </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A34" t="s">
         <v>78</v>
       </c>
@@ -4864,7 +4930,7 @@
         <v>4.6453500000000002E-2</v>
       </c>
     </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A35" t="s">
         <v>80</v>
       </c>
@@ -4908,7 +4974,7 @@
         <v>3.1199999999999999E-4</v>
       </c>
     </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A36" t="s">
         <v>81</v>
       </c>
@@ -4955,7 +5021,7 @@
         <v>1.8806199999999999E-2</v>
       </c>
     </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" t="s">
         <v>82</v>
       </c>
@@ -5002,7 +5068,7 @@
         <v>8.0712000000000006E-3</v>
       </c>
     </row>
-    <row r="38" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" t="s">
         <v>84</v>
       </c>
@@ -5046,7 +5112,7 @@
         <v>9.990000000000001E-4</v>
       </c>
     </row>
-    <row r="39" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>85</v>
       </c>
@@ -5093,7 +5159,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A40" t="s">
         <v>87</v>
       </c>
@@ -5137,7 +5203,7 @@
         <v>8.7625800000000004E-2</v>
       </c>
     </row>
-    <row r="41" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A41" t="s">
         <v>89</v>
       </c>
@@ -5181,7 +5247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A42" t="s">
         <v>90</v>
       </c>
@@ -5225,7 +5291,7 @@
         <v>6.0039999999999996E-4</v>
       </c>
     </row>
-    <row r="43" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A43" t="s">
         <v>91</v>
       </c>
@@ -5269,7 +5335,7 @@
         <v>7.6000000000000004E-4</v>
       </c>
     </row>
-    <row r="44" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
         <v>92</v>
       </c>
@@ -5313,7 +5379,7 @@
         <v>3.5359999999999998E-4</v>
       </c>
     </row>
-    <row r="45" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A45" t="s">
         <v>93</v>
       </c>
@@ -5368,27 +5434,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:P5"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="12.453125" customWidth="1"/>
-    <col min="2" max="2" width="11.81640625" customWidth="1"/>
-    <col min="3" max="3" width="12.26953125" customWidth="1"/>
-    <col min="4" max="4" width="14.81640625" customWidth="1"/>
-    <col min="5" max="5" width="18.6328125" customWidth="1"/>
-    <col min="6" max="6" width="14.453125" customWidth="1"/>
-    <col min="7" max="7" width="22.26953125" customWidth="1"/>
-    <col min="8" max="8" width="16.6328125" customWidth="1"/>
-    <col min="9" max="9" width="20.7265625" customWidth="1"/>
-    <col min="10" max="10" width="18.26953125" customWidth="1"/>
-    <col min="11" max="11" width="20.81640625" customWidth="1"/>
-    <col min="12" max="12" width="18.26953125" customWidth="1"/>
-    <col min="13" max="13" width="20.453125" customWidth="1"/>
-    <col min="14" max="14" width="23.453125" customWidth="1"/>
-    <col min="15" max="15" width="27.36328125" customWidth="1"/>
-    <col min="16" max="16" width="15.1796875" customWidth="1"/>
+    <col min="1" max="1" width="12.47265625" customWidth="1"/>
+    <col min="2" max="2" width="11.7890625" customWidth="1"/>
+    <col min="3" max="3" width="12.26171875" customWidth="1"/>
+    <col min="4" max="4" width="14.7890625" customWidth="1"/>
+    <col min="5" max="5" width="18.62890625" customWidth="1"/>
+    <col min="6" max="6" width="14.47265625" customWidth="1"/>
+    <col min="7" max="7" width="22.26171875" customWidth="1"/>
+    <col min="8" max="8" width="16.62890625" customWidth="1"/>
+    <col min="9" max="9" width="20.734375" customWidth="1"/>
+    <col min="10" max="10" width="18.26171875" customWidth="1"/>
+    <col min="11" max="11" width="20.7890625" customWidth="1"/>
+    <col min="12" max="12" width="18.26171875" customWidth="1"/>
+    <col min="13" max="13" width="20.47265625" customWidth="1"/>
+    <col min="14" max="14" width="23.47265625" customWidth="1"/>
+    <col min="15" max="15" width="27.3671875" customWidth="1"/>
+    <col min="16" max="16" width="15.15625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -5438,7 +5504,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" t="s">
         <v>36</v>
       </c>
@@ -5485,7 +5551,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="3" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" t="s">
         <v>39</v>
       </c>
@@ -5532,7 +5598,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="4" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -5579,7 +5645,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="5" spans="1:16" ht="29" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:16" ht="28.8" x14ac:dyDescent="0.55000000000000004">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -5637,15 +5703,15 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D23"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="24" customWidth="1"/>
-    <col min="2" max="2" width="32.08984375" customWidth="1"/>
-    <col min="3" max="3" width="19.453125" customWidth="1"/>
-    <col min="4" max="4" width="28.36328125" customWidth="1"/>
+    <col min="2" max="2" width="32.1015625" customWidth="1"/>
+    <col min="3" max="3" width="19.47265625" customWidth="1"/>
+    <col min="4" max="4" width="28.3671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>95</v>
       </c>
@@ -5653,7 +5719,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>97</v>
       </c>
@@ -5661,7 +5727,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>98</v>
       </c>
@@ -5669,7 +5735,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>100</v>
       </c>
@@ -5677,7 +5743,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C8" s="6" t="s">
         <v>115</v>
       </c>
@@ -5685,12 +5751,12 @@
         <v>116</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="6" t="s">
         <v>1</v>
       </c>
@@ -5704,161 +5770,161 @@
         <v>14</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>17</v>
       </c>
       <c r="B11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="7">
         <v>0.55196216997500014</v>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="7">
         <v>0.54975048553055572</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B12" t="s">
         <v>28</v>
       </c>
-      <c r="C12" s="9">
+      <c r="C12" s="8">
         <v>0.37422907173333342</v>
       </c>
-      <c r="D12" s="9">
+      <c r="D12" s="8">
         <v>0.37422907173333342</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" t="s">
         <v>73</v>
       </c>
-      <c r="C13" s="9">
+      <c r="C13" s="8">
         <v>3.2960999999999997E-2</v>
       </c>
-      <c r="D13" s="9">
+      <c r="D13" s="8">
         <v>3.2960999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B14" t="s">
         <v>79</v>
       </c>
-      <c r="C14" s="9">
+      <c r="C14" s="8">
         <v>6.5571699999999997E-2</v>
       </c>
-      <c r="D14" s="9">
+      <c r="D14" s="8">
         <v>6.5571699999999997E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B15" t="s">
         <v>83</v>
       </c>
-      <c r="C15" s="9">
+      <c r="C15" s="8">
         <v>9.0702000000000005E-3</v>
       </c>
-      <c r="D15" s="9">
+      <c r="D15" s="8">
         <v>9.0702000000000005E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" t="s">
         <v>33</v>
       </c>
       <c r="B16" t="s">
         <v>34</v>
       </c>
-      <c r="C16" s="8">
+      <c r="C16" s="7">
         <v>1.578702681226388</v>
       </c>
-      <c r="D16" s="8">
+      <c r="D16" s="7">
         <v>1.578702681226388</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B17" t="s">
         <v>52</v>
       </c>
-      <c r="C17" s="8">
+      <c r="C17" s="7">
         <v>0.9030765003222252</v>
       </c>
-      <c r="D17" s="8">
+      <c r="D17" s="7">
         <v>0.9030765003222252</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B18" t="s">
         <v>55</v>
       </c>
-      <c r="C18" s="8">
+      <c r="C18" s="7">
         <v>0.69727071762222104</v>
       </c>
-      <c r="D18" s="8">
+      <c r="D18" s="7">
         <v>0.69727071762222104</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B19" t="s">
         <v>69</v>
       </c>
-      <c r="C19" s="8">
+      <c r="C19" s="7">
         <v>0.69416757355000314</v>
       </c>
-      <c r="D19" s="8">
+      <c r="D19" s="7">
         <v>0.69416757355000314</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A20" t="s">
         <v>40</v>
       </c>
       <c r="B20" t="s">
         <v>41</v>
       </c>
-      <c r="C20" s="8">
+      <c r="C20" s="7">
         <v>0.56643978095000014</v>
       </c>
-      <c r="D20" s="8">
+      <c r="D20" s="7">
         <v>0.56643978095000014</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B21" t="s">
         <v>86</v>
       </c>
-      <c r="C21" s="9">
+      <c r="C21" s="8">
         <v>9.1038581856961995E-2</v>
       </c>
-      <c r="D21" s="9">
+      <c r="D21" s="8">
         <v>9.0854749856962E-2</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" t="s">
         <v>58</v>
       </c>
       <c r="B22" t="s">
         <v>59</v>
       </c>
-      <c r="C22" s="8">
+      <c r="C22" s="7">
         <v>4.1212790261145837</v>
       </c>
-      <c r="D22" s="10">
+      <c r="D22" s="9">
         <v>4.1212790261145837</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A23" t="s">
         <v>63</v>
       </c>
       <c r="B23" t="s">
         <v>64</v>
       </c>
-      <c r="C23" s="8">
+      <c r="C23" s="7">
         <v>0.67515460920750847</v>
       </c>
-      <c r="D23" s="8">
+      <c r="D23" s="7">
         <v>0.67515460920750847</v>
       </c>
     </row>
@@ -5870,15 +5936,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:D51"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
-    <col min="1" max="1" width="24.6328125" customWidth="1"/>
-    <col min="2" max="2" width="33.7265625" customWidth="1"/>
-    <col min="3" max="3" width="31.36328125" customWidth="1"/>
-    <col min="4" max="4" width="29.54296875" customWidth="1"/>
+    <col min="1" max="1" width="24.62890625" customWidth="1"/>
+    <col min="2" max="2" width="33.734375" customWidth="1"/>
+    <col min="3" max="3" width="31.3671875" customWidth="1"/>
+    <col min="4" max="4" width="29.5234375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="2" t="s">
         <v>102</v>
       </c>
@@ -5892,7 +5958,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="3" t="s">
         <v>106</v>
       </c>
@@ -5906,7 +5972,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>107</v>
       </c>
@@ -5920,7 +5986,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A4" s="5" t="s">
         <v>111</v>
       </c>
@@ -5934,7 +6000,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A8" s="6" t="s">
         <v>11</v>
       </c>
@@ -5945,12 +6011,12 @@
         <v>15</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="C9" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="6" t="s">
         <v>1</v>
       </c>
@@ -5961,72 +6027,68 @@
         <v>38</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A11" t="s">
         <v>33</v>
       </c>
       <c r="B11" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="11">
         <v>56.548749999999998</v>
       </c>
-      <c r="D11" s="7"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A12" t="s">
         <v>40</v>
       </c>
       <c r="B12" t="s">
         <v>41</v>
       </c>
-      <c r="C12" s="7">
+      <c r="C12" s="11">
         <v>326.72611111111098</v>
       </c>
-      <c r="D12" s="7"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="B13" t="s">
         <v>86</v>
       </c>
-      <c r="C13" s="7">
+      <c r="C13" s="11">
         <v>21.1</v>
       </c>
-      <c r="D13" s="7"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.55000000000000004">
       <c r="A14" t="s">
         <v>63</v>
       </c>
       <c r="B14" t="s">
         <v>64</v>
       </c>
-      <c r="C14" s="7">
+      <c r="C14" s="11">
         <v>188.495833333333</v>
       </c>
-      <c r="D14" s="7"/>
-    </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.35">
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A30" s="2" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A31" s="3" t="s">
         <v>97</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.55000000000000004">
       <c r="A32" s="4" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A33" s="5" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A37" s="6" t="s">
         <v>12</v>
       </c>
@@ -6034,7 +6096,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A38" s="6" t="s">
         <v>1</v>
       </c>
@@ -6045,122 +6107,122 @@
         <v>19</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A39" t="s">
         <v>17</v>
       </c>
       <c r="B39" t="s">
         <v>18</v>
       </c>
-      <c r="C39">
+      <c r="C39" s="10">
         <v>0.55196216997500014</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B40" t="s">
         <v>28</v>
       </c>
-      <c r="C40">
+      <c r="C40" s="10">
         <v>0.37422907173333342</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B41" t="s">
         <v>73</v>
       </c>
-      <c r="C41">
+      <c r="C41" s="10">
         <v>3.2960999999999997E-2</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B42" t="s">
         <v>79</v>
       </c>
-      <c r="C42">
+      <c r="C42" s="10">
         <v>6.5571699999999997E-2</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B43" t="s">
         <v>83</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="10">
         <v>9.0702000000000005E-3</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A44" t="s">
         <v>33</v>
       </c>
       <c r="B44" t="s">
         <v>34</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="10">
         <v>1.578702681226388</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B45" t="s">
         <v>52</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="10">
         <v>0.9030765003222252</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B46" t="s">
         <v>55</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="10">
         <v>0.69727071762222104</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B47" t="s">
         <v>69</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="10">
         <v>0.69416757355000314</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A48" t="s">
         <v>40</v>
       </c>
       <c r="B48" t="s">
         <v>41</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="10">
         <v>0.56643978095000014</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="B49" t="s">
         <v>86</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="10">
         <v>9.1038581856961995E-2</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A50" t="s">
         <v>58</v>
       </c>
       <c r="B50" t="s">
         <v>59</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="10">
         <v>4.1212790261145837</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.55000000000000004">
       <c r="A51" t="s">
         <v>63</v>
       </c>
       <c r="B51" t="s">
         <v>64</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="10">
         <v>0.67515460920750847</v>
       </c>
     </row>

</xml_diff>